<commit_message>
Initial CQVIP working prototype
</commit_message>
<xml_diff>
--- a/Traceability_Matrix.xlsx
+++ b/Traceability_Matrix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,27 +461,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>URS-001</t>
+          <t>URS-101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The washer shall complete a validated cleaning cycle.</t>
+          <t>The washer shall alarm upon cycle failure.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cleaning</t>
+          <t>Alarm</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OQ / PQ</t>
+          <t>OQ</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>OQ-001, FAT-001, SAT-001, IQ-001</t>
+          <t>OQ-001, IQ-001, FAT-001, SAT-001</t>
         </is>
       </c>
     </row>
@@ -508,22 +508,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The washer shall alarm upon cycle failure.</t>
+          <t>The washer shall complete a validated cleaning cycle.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Alarm</t>
+          <t>Cleaning</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OQ</t>
+          <t>OQ / PQ</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -541,12 +541,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The washer shall record cycle data.</t>
+          <t>The washer shall alarm upon cycle failure.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Data Integrity</t>
+          <t>Alarm</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CSV / OQ</t>
+          <t>OQ</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -574,22 +574,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The system shall maintain pressure during operation.</t>
+          <t>The washer shall record cycle data.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Environmental</t>
+          <t>Data Integrity</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OQ</t>
+          <t>CSV / OQ</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -607,17 +607,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The safety interlock shall prevent unsafe operation.</t>
+          <t>The system shall maintain pressure during operation.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Environmental</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -640,30 +640,261 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>The safety interlock shall prevent unsafe operation.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OQ</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>URS-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>The operator shall complete training before use.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>SOP / Training</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>URS-001</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The washer shall complete a validated cleaning cycle.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Cleaning</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OQ / PQ</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>URS-002</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>The washer shall alarm upon cycle failure.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Alarm</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OQ</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>URS-003</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>The washer shall record cycle data.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Data Integrity</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CSV / OQ</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>URS-004</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The system shall maintain pressure during operation.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>OQ</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>URS-005</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>The safety interlock shall prevent unsafe operation.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>OQ</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>URS-006</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>The operator shall complete training before use.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SOP / Training</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>